<commit_message>
seprated query builder for apps
</commit_message>
<xml_diff>
--- a/TestCases/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
+++ b/TestCases/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -779,12 +779,112 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>GeneticAnalysisTab</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Compare Genetic Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>multi_function</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>TreatmentTab</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Compare Treatments</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>multi_function</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>TreatmentRespTab</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Compare Treatment Response</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>multi_function</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>SurvivalTab</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Compare Survival</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>multi_function</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>SamplesTab</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Compare Samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>multi_function</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>FilesTab</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Compare Files (Explore Files)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
revert additional tab from code
</commit_message>
<xml_diff>
--- a/TestCases/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
+++ b/TestCases/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -779,112 +779,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>GeneticAnalysisTab</t>
+          <t>SamplesTab</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Compare Genetic Analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>14</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>multi_function</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>TreatmentTab</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Compare Treatments</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>15</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>multi_function</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>TreatmentRespTab</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Compare Treatment Response</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>16</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>multi_function</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>SurvivalTab</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Compare Survival</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>17</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>multi_function</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>SamplesTab</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
           <t>Compare Samples</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>18</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>multi_function</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>FilesTab</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Compare Files (Explore Files)</t>
         </is>
       </c>
     </row>

</xml_diff>